<commit_message>
updated logos, exercises for scheduling, and overview
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0576BC5-D169-CA46-A695-7291F90758DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD4F5AD-CC1C-EF49-83BA-5EF4239F8470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="113">
   <si>
     <t>Lecture</t>
   </si>
@@ -365,22 +365,19 @@
     <t>Comments</t>
   </si>
   <si>
-    <t xml:space="preserve">Being the last part, there were 2 variants, one that said "cut". This cut one, the one I picked, is the one that did not point to the questionnare at the end. Should check the final part of other videos too and maybe cut </t>
-  </si>
-  <si>
-    <t>No pointing to questionnaire here, so good</t>
-  </si>
-  <si>
     <t>The slides contain the lecture number and they should not</t>
   </si>
   <si>
-    <t>These slides have changed, they now contain the new file system structure. Also, is FAT still used actually?</t>
-  </si>
-  <si>
     <t>Containers</t>
   </si>
   <si>
     <t>to be recorded</t>
+  </si>
+  <si>
+    <t>to be recorded. Would be nice to add slides/video on different sile systems too (FAT…)</t>
+  </si>
+  <si>
+    <t>There are no questions at the end of this deck</t>
   </si>
 </sst>
 </file>
@@ -428,10 +425,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -911,9 +909,6 @@
       <c r="H5" t="s">
         <v>14</v>
       </c>
-      <c r="I5" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -1096,9 +1091,6 @@
       <c r="H12" t="s">
         <v>14</v>
       </c>
-      <c r="I12" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
@@ -1204,7 +1196,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>12</v>
       </c>
@@ -1230,7 +1222,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>12</v>
       </c>
@@ -1256,7 +1248,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>12</v>
       </c>
@@ -1282,7 +1274,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>12</v>
       </c>
@@ -1307,11 +1299,8 @@
       <c r="H20" t="s">
         <v>14</v>
       </c>
-      <c r="I20" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>13</v>
       </c>
@@ -1337,7 +1326,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
@@ -1363,7 +1352,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
@@ -1389,7 +1378,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -1415,7 +1404,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>13</v>
       </c>
@@ -1441,7 +1430,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>13</v>
       </c>
@@ -1467,7 +1456,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>13</v>
       </c>
@@ -1492,11 +1481,8 @@
       <c r="H27" t="s">
         <v>14</v>
       </c>
-      <c r="I27" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>20</v>
       </c>
@@ -1522,7 +1508,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>20</v>
       </c>
@@ -1548,7 +1534,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>20</v>
       </c>
@@ -1574,7 +1560,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>20</v>
       </c>
@@ -1600,7 +1586,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>20</v>
       </c>
@@ -1677,8 +1663,8 @@
       <c r="H34" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I34" t="s">
-        <v>109</v>
+      <c r="I34" s="3" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
@@ -1914,9 +1900,6 @@
       <c r="H43" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I43" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -2099,9 +2082,6 @@
       <c r="H50" t="s">
         <v>14</v>
       </c>
-      <c r="I50" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
@@ -2284,9 +2264,6 @@
       <c r="H57" t="s">
         <v>14</v>
       </c>
-      <c r="I57" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
@@ -2314,7 +2291,7 @@
         <v>14</v>
       </c>
       <c r="I58" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
@@ -2475,11 +2452,8 @@
       <c r="H64" t="s">
         <v>14</v>
       </c>
-      <c r="I64" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>57</v>
       </c>
@@ -2505,7 +2479,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>57</v>
       </c>
@@ -2531,7 +2505,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>57</v>
       </c>
@@ -2557,7 +2531,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>57</v>
       </c>
@@ -2583,7 +2557,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>57</v>
       </c>
@@ -2609,7 +2583,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>57</v>
       </c>
@@ -2634,11 +2608,8 @@
       <c r="H70" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I70" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>95</v>
       </c>
@@ -2664,7 +2635,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>95</v>
       </c>
@@ -2690,7 +2661,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>95</v>
       </c>
@@ -2716,7 +2687,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>95</v>
       </c>
@@ -2742,7 +2713,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>95</v>
       </c>
@@ -2768,7 +2739,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>95</v>
       </c>
@@ -2794,7 +2765,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>95</v>
       </c>
@@ -2820,7 +2791,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>95</v>
       </c>
@@ -2845,11 +2816,8 @@
       <c r="H78" t="s">
         <v>14</v>
       </c>
-      <c r="I78" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>96</v>
       </c>
@@ -2875,7 +2843,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>96</v>
       </c>
@@ -3056,9 +3024,6 @@
       <c r="H86" t="s">
         <v>14</v>
       </c>
-      <c r="I86" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
@@ -3071,10 +3036,10 @@
         <v>55</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="I87" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed logo, moved exercises, updated overview for lecture on memory management
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD4F5AD-CC1C-EF49-83BA-5EF4239F8470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2792D331-CE36-7544-BDD7-7A662F1E2311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="114">
   <si>
     <t>Lecture</t>
   </si>
@@ -378,6 +378,9 @@
   </si>
   <si>
     <t>There are no questions at the end of this deck</t>
+  </si>
+  <si>
+    <t>Exercises to be checked</t>
   </si>
 </sst>
 </file>
@@ -425,11 +428,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1900,6 +1904,9 @@
       <c r="H43" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I43" s="3" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -2082,6 +2089,7 @@
       <c r="H50" t="s">
         <v>14</v>
       </c>
+      <c r="I50" s="4"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
@@ -2264,6 +2272,9 @@
       <c r="H57" t="s">
         <v>14</v>
       </c>
+      <c r="I57" s="3" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
@@ -2452,8 +2463,11 @@
       <c r="H64" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I64" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>57</v>
       </c>
@@ -2479,7 +2493,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>57</v>
       </c>
@@ -2505,7 +2519,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>57</v>
       </c>
@@ -2531,7 +2545,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>57</v>
       </c>
@@ -2557,7 +2571,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>57</v>
       </c>
@@ -2583,7 +2597,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>57</v>
       </c>
@@ -2608,8 +2622,11 @@
       <c r="H70" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I70" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>95</v>
       </c>
@@ -2635,7 +2652,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>95</v>
       </c>
@@ -2661,7 +2678,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>95</v>
       </c>
@@ -2687,7 +2704,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>95</v>
       </c>
@@ -2713,7 +2730,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>95</v>
       </c>
@@ -2739,7 +2756,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>95</v>
       </c>
@@ -2765,7 +2782,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>95</v>
       </c>
@@ -2791,7 +2808,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>95</v>
       </c>
@@ -2816,8 +2833,11 @@
       <c r="H78" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I78" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>96</v>
       </c>
@@ -2843,7 +2863,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>96</v>
       </c>
@@ -3023,6 +3043,9 @@
       </c>
       <c r="H86" t="s">
         <v>14</v>
+      </c>
+      <c r="I86" s="3" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
changed logo, moved exercises, updated overview for lecture on virtual memory
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2792D331-CE36-7544-BDD7-7A662F1E2311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8ADE78F-749C-D84F-A08A-11F33FEA2F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="114">
   <si>
     <t>Lecture</t>
   </si>
@@ -2272,9 +2272,7 @@
       <c r="H57" t="s">
         <v>14</v>
       </c>
-      <c r="I57" s="3" t="s">
-        <v>113</v>
-      </c>
+      <c r="I57" s="4"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">

</xml_diff>

<commit_message>
changed logo, moved exercises, updated overview for lecture on file systems
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8ADE78F-749C-D84F-A08A-11F33FEA2F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42091E6E-8723-0747-B741-93E96CD15D44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="113">
   <si>
     <t>Lecture</t>
   </si>
@@ -363,9 +363,6 @@
   </si>
   <si>
     <t>Comments</t>
-  </si>
-  <si>
-    <t>The slides contain the lecture number and they should not</t>
   </si>
   <si>
     <t>Containers</t>
@@ -1668,7 +1665,7 @@
         <v>14</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
@@ -1905,7 +1902,7 @@
         <v>14</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
@@ -2299,9 +2296,6 @@
       <c r="H58" t="s">
         <v>14</v>
       </c>
-      <c r="I58" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
@@ -2381,7 +2375,7 @@
         <v>14</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
@@ -2461,9 +2455,7 @@
       <c r="H64" t="s">
         <v>14</v>
       </c>
-      <c r="I64" s="3" t="s">
-        <v>113</v>
-      </c>
+      <c r="I64" s="4"/>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
@@ -2621,7 +2613,7 @@
         <v>14</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
@@ -2832,7 +2824,7 @@
         <v>14</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
@@ -3043,7 +3035,7 @@
         <v>14</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
@@ -3057,10 +3049,10 @@
         <v>55</v>
       </c>
       <c r="D87" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="I87" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="I87" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed logo, moved exercises, updated overview for lecture on security
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42091E6E-8723-0747-B741-93E96CD15D44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877E19D3-15B1-374D-816A-9959B7FF8B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -425,12 +425,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2086,7 +2085,7 @@
       <c r="H50" t="s">
         <v>14</v>
       </c>
-      <c r="I50" s="4"/>
+      <c r="I50" s="1"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
@@ -2269,7 +2268,7 @@
       <c r="H57" t="s">
         <v>14</v>
       </c>
-      <c r="I57" s="4"/>
+      <c r="I57" s="1"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
@@ -2455,7 +2454,7 @@
       <c r="H64" t="s">
         <v>14</v>
       </c>
-      <c r="I64" s="4"/>
+      <c r="I64" s="1"/>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
@@ -2613,7 +2612,7 @@
         <v>14</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
changed logo, moved exercises, updated overview for lecture on I/O systems
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877E19D3-15B1-374D-816A-9959B7FF8B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4982ED9-1E07-F34E-A60E-00E6D8FF1E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="113">
   <si>
     <t>Lecture</t>
   </si>
@@ -425,11 +425,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2585,6 +2586,9 @@
       <c r="H69" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I69" s="3" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
@@ -2611,9 +2615,6 @@
       <c r="H70" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I70" s="3" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
@@ -2822,9 +2823,7 @@
       <c r="H78" t="s">
         <v>14</v>
       </c>
-      <c r="I78" s="3" t="s">
-        <v>112</v>
-      </c>
+      <c r="I78" s="4"/>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">

</xml_diff>

<commit_message>
changed logo, moved exercises, updated overview for lecture on virtualization
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4982ED9-1E07-F34E-A60E-00E6D8FF1E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E44B56E-F3F8-C545-89DD-84AB4A1B81A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="112">
   <si>
     <t>Lecture</t>
   </si>
@@ -375,9 +375,6 @@
   </si>
   <si>
     <t>There are no questions at the end of this deck</t>
-  </si>
-  <si>
-    <t>Exercises to be checked</t>
   </si>
 </sst>
 </file>
@@ -3033,7 +3030,7 @@
         <v>14</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
added questions synchronization 1
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E44B56E-F3F8-C545-89DD-84AB4A1B81A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E134EFB-3DC6-104E-9D1F-91A0BEA371C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="113">
   <si>
     <t>Lecture</t>
   </si>
@@ -375,6 +375,9 @@
   </si>
   <si>
     <t>There are no questions at the end of this deck</t>
+  </si>
+  <si>
+    <t>It says the fourth edition is OK too, should change that. Most of these slides can actually go I think</t>
   </si>
 </sst>
 </file>
@@ -829,6 +832,9 @@
       <c r="H2" t="s">
         <v>14</v>
       </c>
+      <c r="I2" s="2" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1661,9 +1667,7 @@
       <c r="H34" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I34" s="3" t="s">
-        <v>111</v>
-      </c>
+      <c r="I34" s="4"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
@@ -2820,7 +2824,7 @@
       <c r="H78" t="s">
         <v>14</v>
       </c>
-      <c r="I78" s="4"/>
+      <c r="I78" s="1"/>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">

</xml_diff>

<commit_message>
added missing subtitles for scheduling part 07
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E134EFB-3DC6-104E-9D1F-91A0BEA371C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{591BC57C-CF56-5841-AA8A-6E9713C344C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -425,12 +425,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1667,7 +1666,7 @@
       <c r="H34" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I34" s="4"/>
+      <c r="I34" s="1"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">

</xml_diff>

<commit_message>
added links to youtube playlists
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{591BC57C-CF56-5841-AA8A-6E9713C344C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25731C50-0D1F-BF45-9107-E550BB687F62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="114">
   <si>
     <t>Lecture</t>
   </si>
@@ -378,6 +378,9 @@
   </si>
   <si>
     <t>It says the fourth edition is OK too, should change that. Most of these slides can actually go I think</t>
+  </si>
+  <si>
+    <t>should check cutting in the beginning</t>
   </si>
 </sst>
 </file>
@@ -1930,6 +1933,9 @@
       <c r="H44" t="s">
         <v>14</v>
       </c>
+      <c r="I44" s="2" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
@@ -1956,6 +1962,9 @@
       <c r="H45" t="s">
         <v>14</v>
       </c>
+      <c r="I45" s="2" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -1982,6 +1991,9 @@
       <c r="H46" t="s">
         <v>14</v>
       </c>
+      <c r="I46" s="2" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
@@ -2008,6 +2020,9 @@
       <c r="H47" t="s">
         <v>14</v>
       </c>
+      <c r="I47" s="2" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
@@ -2034,6 +2049,9 @@
       <c r="H48" t="s">
         <v>14</v>
       </c>
+      <c r="I48" s="2" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
@@ -2059,6 +2077,9 @@
       </c>
       <c r="H49" t="s">
         <v>14</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added video on virtualization / containers
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25731C50-0D1F-BF45-9107-E550BB687F62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5E73E7-6C48-DE49-9C73-77F42A3316D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="112">
   <si>
     <t>Lecture</t>
   </si>
@@ -368,19 +368,13 @@
     <t>Containers</t>
   </si>
   <si>
-    <t>to be recorded</t>
-  </si>
-  <si>
-    <t>to be recorded. Would be nice to add slides/video on different sile systems too (FAT…)</t>
-  </si>
-  <si>
     <t>There are no questions at the end of this deck</t>
   </si>
   <si>
-    <t>It says the fourth edition is OK too, should change that. Most of these slides can actually go I think</t>
-  </si>
-  <si>
     <t>should check cutting in the beginning</t>
+  </si>
+  <si>
+    <t>Would be nice to add slides/video on different sile systems too (FAT…)</t>
   </si>
 </sst>
 </file>
@@ -428,11 +422,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -834,9 +829,7 @@
       <c r="H2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>112</v>
-      </c>
+      <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1905,7 +1898,7 @@
         <v>14</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
@@ -1934,7 +1927,7 @@
         <v>14</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
@@ -1963,7 +1956,7 @@
         <v>14</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
@@ -1992,7 +1985,7 @@
         <v>14</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
@@ -2021,7 +2014,7 @@
         <v>14</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
@@ -2050,7 +2043,7 @@
         <v>14</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
@@ -2079,7 +2072,7 @@
         <v>14</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
@@ -2396,7 +2389,7 @@
         <v>14</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
@@ -2608,7 +2601,7 @@
         <v>14</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
@@ -3054,7 +3047,7 @@
         <v>14</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
@@ -3070,9 +3063,7 @@
       <c r="D87" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="I87" s="2" t="s">
-        <v>109</v>
-      </c>
+      <c r="I87" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
added questions to security slides
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5E73E7-6C48-DE49-9C73-77F42A3316D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9AA033-5198-7F41-8B4C-772BD4669E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="112">
   <si>
     <t>Lecture</t>
   </si>
@@ -427,7 +427,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -829,7 +829,6 @@
       <c r="H2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -2600,9 +2599,7 @@
       <c r="H69" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I69" s="3" t="s">
-        <v>109</v>
-      </c>
+      <c r="I69" s="4"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
@@ -3063,7 +3060,6 @@
       <c r="D87" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="I87" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Added questions for Virtualization lecture
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9AA033-5198-7F41-8B4C-772BD4669E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22526495-5FF6-BD4F-AC47-3CD9A23E4F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="112">
   <si>
     <t>Lecture</t>
   </si>
@@ -2599,7 +2599,7 @@
       <c r="H69" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I69" s="4"/>
+      <c r="I69" s="1"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
@@ -3043,9 +3043,7 @@
       <c r="H86" t="s">
         <v>14</v>
       </c>
-      <c r="I86" s="3" t="s">
-        <v>109</v>
-      </c>
+      <c r="I86" s="4"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">

</xml_diff>

<commit_message>
polished introduction to OS slides
Most important thing: clarified part on setting up interrupts/handlers on start up (slide 18) clarifying priviledge instructions are hardware defined
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinmas/repositories/os_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22526495-5FF6-BD4F-AC47-3CD9A23E4F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98192B15-0A4C-594F-9D18-ACFAD5D5BF59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17020" xr2:uid="{67D7C5C9-BFD9-9043-B236-4D7F530C133A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="112">
   <si>
     <t>Lecture</t>
   </si>
@@ -422,12 +422,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -907,6 +906,9 @@
       <c r="H5" t="s">
         <v>14</v>
       </c>
+      <c r="I5" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -3043,7 +3045,7 @@
       <c r="H86" t="s">
         <v>14</v>
       </c>
-      <c r="I86" s="4"/>
+      <c r="I86" s="1"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">

</xml_diff>